<commit_message>
chore: 差分表補回尼莫第 6 張 ＋ -1507 的 cache-buster 收尾
· 美術 813ff7f 救回 `Nemo_SI_dual.webp` ⇒ 表重跑（尼莫 5→6、差分 329→330）。
· ⚠ `bust.py --bump` 會動**四支檔**（config.js／index.html／flight/index.html／
  modules/story.js 的 KERB_V），-1507 那兩個 commit 我只帶到前兩支 ——
  漏掉的那兩支正是**飛行頁自己的 `?v=`**，留著的話飛行頁會一直吃 1505 的快取
  （§6 的 -1461：版本號沒動＝那一版送不到玩家手上，這是它的另一半）。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/SI/_SI_差分總表.xlsx
+++ b/resources/SI/_SI_差分總表.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安雅" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="賽西莉" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="璐娜莉亞" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="蘿芮" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="尼莫" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="尼莫" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="蘿芮" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="托爾斯坦" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阿瑞尼斯" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城鎮店主 NPC" sheetId="11" state="visible" r:id="rId11"/>
@@ -8248,6 +8248,31 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1333500" cy="1333500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -14759,7 +14784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D105"/>
+  <dimension ref="A1:D106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15331,7 +15356,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Nemo_SI_front.webp</t>
+          <t>Nemo_SI_dual.webp</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -15353,7 +15378,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Nemo_SI_happy.webp</t>
+          <t>Nemo_SI_front.webp</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -15375,7 +15400,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Nemo_SI_surprise.webp</t>
+          <t>Nemo_SI_happy.webp</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -15392,12 +15417,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Nouvelle_Nun</t>
+          <t>Nemo</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Nouvelle_Nun_SI_front.webp</t>
+          <t>Nemo_SI_surprise.webp</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -15414,12 +15439,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nouvelle</t>
+          <t>Nouvelle_Nun</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Nouvelle_SI_Scared.webp</t>
+          <t>Nouvelle_Nun_SI_front.webp</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -15441,7 +15466,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Nouvelle_SI_back.webp</t>
+          <t>Nouvelle_SI_Scared.webp</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -15463,7 +15488,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Nouvelle_SI_bye.webp</t>
+          <t>Nouvelle_SI_back.webp</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -15485,7 +15510,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Nouvelle_SI_expainsweat.webp</t>
+          <t>Nouvelle_SI_bye.webp</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -15507,7 +15532,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Nouvelle_SI_meetagain.webp</t>
+          <t>Nouvelle_SI_expainsweat.webp</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -15529,7 +15554,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Nouvelle_SI_reliefbreath.webp</t>
+          <t>Nouvelle_SI_meetagain.webp</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -15551,7 +15576,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Nouvelle_SI_side.webp</t>
+          <t>Nouvelle_SI_reliefbreath.webp</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -15568,12 +15593,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>RennaSorana</t>
+          <t>Nouvelle</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>RennaSorana_SI_annoyedC.webp</t>
+          <t>Nouvelle_SI_side.webp</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -15595,7 +15620,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>RennaSorana_SI_annoyedD.webp</t>
+          <t>RennaSorana_SI_annoyedC.webp</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -15612,12 +15637,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Renna</t>
+          <t>RennaSorana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Renna_SI_annoyed.webp</t>
+          <t>RennaSorana_SI_annoyedD.webp</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -15634,12 +15659,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Sorana</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Sorana_SI_drink.webp</t>
+          <t>Renna_SI_annoyed.webp</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -15661,7 +15686,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Sorana_SI_shy.webp</t>
+          <t>Sorana_SI_drink.webp</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -15678,12 +15703,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Torsten</t>
+          <t>Sorana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Torsten_SI_Q.webp</t>
+          <t>Sorana_SI_shy.webp</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -15705,7 +15730,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Torsten_SI_front.webp</t>
+          <t>Torsten_SI_Q.webp</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -15722,12 +15747,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>XAnya</t>
+          <t>Torsten</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>XAnya_SI_front.webp</t>
+          <t>Torsten_SI_front.webp</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -15744,12 +15769,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Gen_Renna</t>
+          <t>XAnya</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>gen_Renna_SI_blushed.webp</t>
+          <t>XAnya_SI_front.webp</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -15766,12 +15791,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Sorana</t>
+          <t>Gen_Renna</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>sorana_SI_Q.webp</t>
+          <t>gen_Renna_SI_blushed.webp</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -15783,22 +15808,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>同差分的另一個版本</t>
+          <t>美術交了沒接線</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>NPC_Grocer</t>
+          <t>Sorana</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>resources/SI/NPC/NPC_Grocer_SI_v2.webp</t>
+          <t>sorana_SI_Q.webp</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>線上跑的是 NPC_Grocer_SI_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
         </is>
       </c>
     </row>
@@ -15815,7 +15840,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>resources/SI/NPC/NPC_Grocer_SI_v3.webp</t>
+          <t>resources/SI/NPC/NPC_Grocer_SI_v2.webp</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -15837,7 +15862,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>resources/SI/NPC/NPC_Grocer_SI_v4.webp</t>
+          <t>resources/SI/NPC/NPC_Grocer_SI_v3.webp</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -15859,7 +15884,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>resources/SI/NPC/NPC_Grocer_SI_v5.webp</t>
+          <t>resources/SI/NPC/NPC_Grocer_SI_v4.webp</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -15876,17 +15901,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>NPC_GuildCounter</t>
+          <t>NPC_Grocer</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>resources/SI/NPC/NPC_GuildCounter_SI_v1.webp</t>
+          <t>resources/SI/NPC/NPC_Grocer_SI_v5.webp</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>線上跑的是 NPC_GuildCounter_SI_v5.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 NPC_Grocer_SI_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -15903,7 +15928,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>resources/SI/NPC/NPC_GuildCounter_SI_v3.webp</t>
+          <t>resources/SI/NPC/NPC_GuildCounter_SI_v1.webp</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -15925,7 +15950,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>resources/SI/NPC/NPC_GuildCounter_SI_v4.webp</t>
+          <t>resources/SI/NPC/NPC_GuildCounter_SI_v3.webp</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -15942,17 +15967,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>NPC_Gunsmith</t>
+          <t>NPC_GuildCounter</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>resources/SI/NPC/NPC_Gunsmith_SI_v2.webp</t>
+          <t>resources/SI/NPC/NPC_GuildCounter_SI_v4.webp</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>線上跑的是 NPC_Gunsmith_SI_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 NPC_GuildCounter_SI_v5.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -15969,7 +15994,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>resources/SI/NPC/NPC_Gunsmith_SI_v3.webp</t>
+          <t>resources/SI/NPC/NPC_Gunsmith_SI_v2.webp</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -15991,7 +16016,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>resources/SI/NPC/NPC_Gunsmith_SI_v4.webp</t>
+          <t>resources/SI/NPC/NPC_Gunsmith_SI_v3.webp</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -16013,7 +16038,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>resources/SI/NPC/NPC_Gunsmith_SI_v5.webp</t>
+          <t>resources/SI/NPC/NPC_Gunsmith_SI_v4.webp</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -16030,17 +16055,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>NPC_Gunsmith</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>resources/SI/OLD/cecilie_si_front.png</t>
+          <t>resources/SI/NPC/NPC_Gunsmith_SI_v5.webp</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>線上跑的是 Cecilie_SI_front.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 NPC_Gunsmith_SI_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16057,12 +16082,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>resources/SI/OLD/cecilie_si_lookaside.png</t>
+          <t>resources/SI/OLD/cecilie_si_front.png</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>線上跑的是 Cecilie_SI_lookaside.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Cecilie_SI_front.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16079,12 +16104,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>resources/SI/OLD/cecilie_si_sadback.png</t>
+          <t>resources/SI/OLD/cecilie_si_lookaside.png</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>線上跑的是 Cecilie_SI_sadback.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Cecilie_SI_lookaside.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16101,12 +16126,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>resources/SI/OLD/cecilie_si_smile.png</t>
+          <t>resources/SI/OLD/cecilie_si_sadback.png</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>線上跑的是 Cecilie_SI_smile.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Cecilie_SI_sadback.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16123,12 +16148,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>resources/SI/OLD/cecilie_si_tease.png</t>
+          <t>resources/SI/OLD/cecilie_si_smile.png</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>線上跑的是 Cecilie_SI_tease.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Cecilie_SI_smile.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16145,12 +16170,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>resources/SI/OLD/cecilie_si_upset.png</t>
+          <t>resources/SI/OLD/cecilie_si_tease.png</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>線上跑的是 Cecilie_SI_upset.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Cecilie_SI_tease.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16162,17 +16187,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Renna</t>
+          <t>Cecilie</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_Pause.webp</t>
+          <t>resources/SI/OLD/cecilie_si_upset.png</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_Pause.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Cecilie_SI_upset.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16189,12 +16214,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_Shout.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_Pause.webp</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_Shout.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_Pause.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16211,12 +16236,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_Surprise.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_Shout.webp</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_Surprise.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_Shout.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16233,12 +16258,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_argue.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_Surprise.webp</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_argue.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_Surprise.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16255,12 +16280,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_arguecute.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_argue.webp</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_arguecute.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_argue.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16277,12 +16302,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_ask.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_arguecute.webp</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_ask.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_arguecute.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16299,12 +16324,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_askserious.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_ask.webp</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_askserious.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_ask.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16321,12 +16346,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_awkwerd.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_askserious.webp</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_awkwerd.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_askserious.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16343,12 +16368,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_blushed.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_awkwerd.webp</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_blushed.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_awkwerd.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16365,12 +16390,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_bow.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_blushed.webp</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_bow.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_blushed.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16387,12 +16412,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_callangry.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_bow.webp</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_callangry.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_bow.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16409,12 +16434,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_chase.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_callangry.webp</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_chase.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_callangry.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16431,12 +16456,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_chase2.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_chase.webp</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_chase2.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_chase.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16453,12 +16478,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_command.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_chase2.webp</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_command.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_chase2.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16475,12 +16500,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_covermouth.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_command.webp</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_covermouth.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_command.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16497,12 +16522,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_cringe.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_covermouth.webp</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_cringe.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_covermouth.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16519,12 +16544,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_curious.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_cringe.webp</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_curious.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_cringe.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16541,12 +16566,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_dying.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_curious.webp</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_dying.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_curious.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16563,12 +16588,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_evalutating.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_dying.webp</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_evalutating.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_dying.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16585,12 +16610,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_evalutatingclosemouth.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_evalutating.webp</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_evalutatingclosemouth.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_evalutating.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16607,12 +16632,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_front.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_evalutatingclosemouth.webp</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_front.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_evalutatingclosemouth.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16629,12 +16654,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_intense.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_front.webp</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_intense.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_front.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16651,12 +16676,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_intense2.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_intense.webp</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_intense2.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_intense.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16673,12 +16698,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_invite.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_intense2.webp</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_invite.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_intense2.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16695,12 +16720,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_lookaway.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_invite.webp</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_lookaway.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_invite.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16717,12 +16742,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_lookawaytalk.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_lookaway.webp</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_lookawaytalk.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_lookaway.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16739,12 +16764,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_lookdown.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_lookawaytalk.webp</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_lookdown.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_lookawaytalk.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16761,12 +16786,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_lookup.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_lookdown.webp</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_lookup.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_lookdown.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16783,12 +16808,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_relief.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_lookup.webp</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_relief.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_lookup.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16805,12 +16830,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_sad.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_relief.webp</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_sad.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_relief.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16827,12 +16852,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_smile.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_sad.webp</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_smile.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_sad.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16849,12 +16874,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_stare.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_smile.webp</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_stare.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_smile.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16871,12 +16896,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_talkserious.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_stare.webp</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_talkserious.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_stare.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16893,12 +16918,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_talkwork.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_talkserious.webp</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_talkwork.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_talkserious.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16915,12 +16940,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_thinking.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_talkwork.webp</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_thinking.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_talkwork.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16937,12 +16962,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_tired.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_thinking.webp</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_tired.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_thinking.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16959,12 +16984,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_upset.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_tired.webp</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_upset.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_tired.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -16981,12 +17006,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_upsetstare.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_upset.webp</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_upsetstare.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_upset.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -17003,12 +17028,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_wake.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_upsetstare.webp</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_wake.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_upsetstare.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -17025,12 +17050,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_watch.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_wake.webp</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_watch.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_wake.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -17047,12 +17072,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>resources/SI/renna_newhair/Renna_SI_worry.webp</t>
+          <t>resources/SI/renna_newhair/Renna_SI_watch.webp</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>線上跑的是 Renna_SI_worry.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 Renna_SI_watch.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -17069,10 +17094,32 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
+          <t>resources/SI/renna_newhair/Renna_SI_worry.webp</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>線上跑的是 Renna_SI_worry.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>同差分的另一個版本</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Renna</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
           <t>resources/SI/renna_newhair/Renna_SI_writting.webp</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
+      <c r="D106" t="inlineStr">
         <is>
           <t>線上跑的是 Renna_SI_writting.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
@@ -26739,7 +26786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26821,13 +26868,13 @@
     <row r="2" ht="111" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Laurie</t>
+          <t>Nemo</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Laurie_SI_crying.webp</t>
+          <t>Nemo_SI_bored.webp</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -26856,20 +26903,20 @@
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>resources/SI/Laurie_SI_crying.webp</t>
+          <t>resources/SI/Nemo_SI_bored.webp</t>
         </is>
       </c>
     </row>
     <row r="3" ht="111" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Laurie</t>
+          <t>Nemo</t>
         </is>
       </c>
       <c r="B3" s="3" t="n"/>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Laurie_SI_dying.webp</t>
+          <t>Nemo_SI_bye.webp</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -26898,20 +26945,20 @@
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>resources/SI/Laurie_SI_dying.webp</t>
+          <t>resources/SI/Nemo_SI_bye.webp</t>
         </is>
       </c>
     </row>
     <row r="4" ht="111" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Laurie</t>
+          <t>Nemo</t>
         </is>
       </c>
       <c r="B4" s="3" t="n"/>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Laurie_SI_front.webp</t>
+          <t>Nemo_SI_dual.webp</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -26940,20 +26987,20 @@
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>resources/SI/Laurie_SI_front.webp</t>
+          <t>resources/SI/Nemo_SI_dual.webp</t>
         </is>
       </c>
     </row>
     <row r="5" ht="111" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Laurie</t>
+          <t>Nemo</t>
         </is>
       </c>
       <c r="B5" s="3" t="n"/>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Laurie_SI_idea.webp</t>
+          <t>Nemo_SI_front.webp</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -26982,20 +27029,20 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>resources/SI/Laurie_SI_idea.webp</t>
+          <t>resources/SI/Nemo_SI_front.webp</t>
         </is>
       </c>
     </row>
     <row r="6" ht="111" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Laurie</t>
+          <t>Nemo</t>
         </is>
       </c>
       <c r="B6" s="3" t="n"/>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Laurie_SI_lookaside.webp</t>
+          <t>Nemo_SI_happy.webp</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -27024,7 +27071,49 @@
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>resources/SI/Laurie_SI_lookaside.webp</t>
+          <t>resources/SI/Nemo_SI_happy.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="111" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Nemo</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Nemo_SI_surprise.webp</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>✘ 未接線</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>估</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>resources/SI/Nemo_SI_surprise.webp</t>
         </is>
       </c>
     </row>
@@ -27122,13 +27211,13 @@
     <row r="2" ht="111" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nemo</t>
+          <t>Laurie</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Nemo_SI_bored.webp</t>
+          <t>Laurie_SI_crying.webp</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -27157,20 +27246,20 @@
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>resources/SI/Nemo_SI_bored.webp</t>
+          <t>resources/SI/Laurie_SI_crying.webp</t>
         </is>
       </c>
     </row>
     <row r="3" ht="111" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Nemo</t>
+          <t>Laurie</t>
         </is>
       </c>
       <c r="B3" s="3" t="n"/>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Nemo_SI_bye.webp</t>
+          <t>Laurie_SI_dying.webp</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -27199,20 +27288,20 @@
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>resources/SI/Nemo_SI_bye.webp</t>
+          <t>resources/SI/Laurie_SI_dying.webp</t>
         </is>
       </c>
     </row>
     <row r="4" ht="111" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Nemo</t>
+          <t>Laurie</t>
         </is>
       </c>
       <c r="B4" s="3" t="n"/>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Nemo_SI_front.webp</t>
+          <t>Laurie_SI_front.webp</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -27241,20 +27330,20 @@
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>resources/SI/Nemo_SI_front.webp</t>
+          <t>resources/SI/Laurie_SI_front.webp</t>
         </is>
       </c>
     </row>
     <row r="5" ht="111" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Nemo</t>
+          <t>Laurie</t>
         </is>
       </c>
       <c r="B5" s="3" t="n"/>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Nemo_SI_happy.webp</t>
+          <t>Laurie_SI_idea.webp</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -27283,20 +27372,20 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>resources/SI/Nemo_SI_happy.webp</t>
+          <t>resources/SI/Laurie_SI_idea.webp</t>
         </is>
       </c>
     </row>
     <row r="6" ht="111" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Nemo</t>
+          <t>Laurie</t>
         </is>
       </c>
       <c r="B6" s="3" t="n"/>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Nemo_SI_surprise.webp</t>
+          <t>Laurie_SI_lookaside.webp</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -27325,7 +27414,7 @@
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>resources/SI/Nemo_SI_surprise.webp</t>
+          <t>resources/SI/Laurie_SI_lookaside.webp</t>
         </is>
       </c>
     </row>

</xml_diff>